<commit_message>
rename and code optimization
</commit_message>
<xml_diff>
--- a/result_kg_reproduce/table_merge/Paper_All_Tables_Merged.xlsx
+++ b/result_kg_reproduce/table_merge/Paper_All_Tables_Merged.xlsx
@@ -2690,7 +2690,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Supplier FE + Src FE+ App FE</t>
+          <t>Supplier FE + Src FE + App FE</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Paid API listings with positive normalized posted prices after cleaning.</t>
+          <t>Final modeling API listings matched to the KG through anonymized product and supplier labels.</t>
         </is>
       </c>
     </row>

</xml_diff>